<commit_message>
Track companies data and pipeline Excel outputs; ignore debug dirs only
- Relax .gitignore: stop ignoring all final_excel/ and final xlsx files
- Ignore companies/**/debug/ for intermediate pipeline artifacts
- Add per-company configs, merged statements, and final_excel/excel workbooks

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/companies/SKHYNIX/SKHYNIX_financial_statements_final.xlsx
+++ b/companies/SKHYNIX/SKHYNIX_financial_statements_final.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Balance Sheet" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Income Statement" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Cash Flow Statement" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balance Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income Statement" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flow Statement" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Balance Sheet'!$A$1:$E$57</definedName>

</xml_diff>